<commit_message>
Fix #REF! and dependencies in cap/floor excel test
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_capfloor.xlsx
+++ b/tests/workbooktests/workbooks/test_capfloor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C544AF4-5931-479E-AA92-0B361A2E8043}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310E900F-15C3-4A5E-AE87-CA79E41EF39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{19136249-26FF-4BA6-AF5B-86DBDAF90384}"/>
+    <workbookView xWindow="3210" yWindow="-20520" windowWidth="27315" windowHeight="17445" xr2:uid="{19136249-26FF-4BA6-AF5B-86DBDAF90384}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabs" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,20 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -470,7 +484,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -486,9 +500,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -526,7 +540,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -632,7 +646,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -774,7 +788,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -783,15 +797,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68E6A32A-A0CE-401D-807A-F91DAD1693EF}">
   <dimension ref="B1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="24" t="s">
         <v>0</v>
       </c>
@@ -800,7 +814,7 @@
       </c>
       <c r="D2" s="27"/>
     </row>
-    <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="25"/>
       <c r="C3" s="6" t="s">
         <v>6</v>
@@ -809,7 +823,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
@@ -820,7 +834,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
@@ -831,7 +845,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>4</v>
       </c>
@@ -842,7 +856,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="5" t="s">
         <v>5</v>
       </c>
@@ -865,15 +879,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B7D6147-A96C-4CC0-B400-4E160714C85B}">
   <dimension ref="A1:E43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="57.85546875" customWidth="1"/>
-    <col min="2" max="2" width="82.140625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="36.85546875" style="8" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" style="8"/>
+    <col min="1" max="1" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="82.109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="36.88671875" style="8" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -881,7 +895,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -890,7 +904,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>10</v>
       </c>
@@ -898,7 +912,7 @@
         <v>46030</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
@@ -906,7 +920,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -915,7 +929,7 @@
       </c>
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
@@ -923,16 +937,16 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B8" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Cap!R8C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>34</v>
       </c>
@@ -941,7 +955,7 @@
         <v>欣[test_capfloor.xlsx]Cap!R9C2USDLibor,A</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>15</v>
       </c>
@@ -950,14 +964,14 @@
         <v>欣[test_capfloor.xlsx]Cap!R10C2IborCoupon,A</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="28"/>
       <c r="B11" s="8" t="str">
         <f>_xll.qlIborCoupon(B6,B7,B4,B6,0,B9)</f>
         <v>欣[test_capfloor.xlsx]Cap!R11C2IborCoupon,A</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="28" t="s">
         <v>35</v>
       </c>
@@ -965,13 +979,13 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="28"/>
       <c r="B13" s="8">
         <v>0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>14</v>
       </c>
@@ -980,7 +994,7 @@
         <v>欣[test_capfloor.xlsx]Cap!R14C2Cap,A</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>16</v>
       </c>
@@ -989,7 +1003,7 @@
         <v>欣[test_capfloor.xlsx]Cap!R15C2CashFlow,A</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>18</v>
       </c>
@@ -998,7 +1012,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>19</v>
       </c>
@@ -1007,7 +1021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>20</v>
       </c>
@@ -1016,7 +1030,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>21</v>
       </c>
@@ -1025,7 +1039,7 @@
         <v>46395</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>22</v>
       </c>
@@ -1034,43 +1048,34 @@
         <v>CAP</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Cap!R21C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="8" t="str">
+      <c r="B22" s="8">
         <f>_xll.qlCapFloorAtmRate(B14,B21)</f>
-        <v xml:space="preserve">TypeError: TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\capfloor.py", line 150, in qlCapFloorAtmRate
-    return capfloor.atmRate(discount_curve)
-           ~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 26935, in atmRate
-    return _QuantLib.CapFloor_atmRate(self, discountCurve)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^^^^^^
-TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3.0038607816972797E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B23" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Cap!R23C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>32</v>
       </c>
@@ -1078,7 +1083,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>25</v>
       </c>
@@ -1087,7 +1092,7 @@
         <v>欣[test_capfloor.xlsx]Cap!R25C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>29</v>
       </c>
@@ -1096,61 +1101,43 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="8" t="str">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="8">
+        <f>_xll.qlInstrumentNPV(B14,B26)</f>
+        <v>5.119883118899232E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B28" s="8" t="str">
+      <c r="B28" s="8">
         <f>_xll.qlCapFloorImpliedVolatility(B14,B27,B23,0.2)</f>
-        <v>Error in arg 2 'price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-': Expected float</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B29" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Cap!R29C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>36</v>
       </c>
       <c r="B30" s="8" t="str">
-        <f>_xll.qlConstantOptionletVolatility(B1,"TARGET","Following",0.2,"actual365Fixed")</f>
+        <f>_xll.qlConstantOptionletVolatility(B2,"TARGET","Following",0.2,"actual365Fixed")</f>
         <v>欣[test_capfloor.xlsx]Cap!R30C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>26</v>
       </c>
@@ -1159,7 +1146,7 @@
         <v>欣[test_capfloor.xlsx]Cap!R31C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
         <v>29</v>
       </c>
@@ -1168,34 +1155,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="8" t="str">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B33" s="8">
+        <f>_xll.qlInstrumentNPV(B14,B32)</f>
+        <v>5.119883118899232E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B34" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Cap!R34C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>32</v>
       </c>
@@ -1203,7 +1181,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>27</v>
       </c>
@@ -1212,7 +1190,7 @@
         <v>欣[test_capfloor.xlsx]Cap!R36C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
         <v>29</v>
       </c>
@@ -1221,34 +1199,34 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>30</v>
       </c>
       <c r="B38" s="8">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v>9.0604094423498536E-5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlInstrumentNPV(B14,B37)</f>
+        <v>5.119883118899232E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B39" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Cap!R39C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B40" s="8" t="str">
-        <f>_xll.qlConstantOptionletVolatility(B1,"TARGET","Following",0.002,"actual365Fixed","normal")</f>
+        <f>_xll.qlConstantOptionletVolatility(B2,"TARGET","Following",0.002,"actual365Fixed","normal")</f>
         <v>欣[test_capfloor.xlsx]Cap!R40C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
         <v>28</v>
       </c>
@@ -1257,7 +1235,7 @@
         <v>欣[test_capfloor.xlsx]Cap!R41C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
         <v>29</v>
       </c>
@@ -1266,13 +1244,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>30</v>
       </c>
       <c r="B43" s="8">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v>9.0604094423498536E-5</v>
+        <f>_xll.qlInstrumentNPV(B14,B42)</f>
+        <v>3.8652710022632174E-3</v>
       </c>
     </row>
   </sheetData>
@@ -1288,15 +1266,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12E17AF-C730-4393-B5FD-E373FB1E4DE1}">
   <dimension ref="A1:E43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="57.85546875" customWidth="1"/>
-    <col min="2" max="2" width="82.140625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="36.85546875" style="8" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" style="8"/>
+    <col min="1" max="1" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="82.109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="36.88671875" style="8" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1304,7 +1282,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1313,7 +1291,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>10</v>
       </c>
@@ -1321,7 +1299,7 @@
         <v>46030</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
@@ -1329,7 +1307,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -1338,7 +1316,7 @@
       </c>
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
@@ -1346,16 +1324,16 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B8" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Floor!R8C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>34</v>
       </c>
@@ -1364,7 +1342,7 @@
         <v>欣[test_capfloor.xlsx]Floor!R9C2USDLibor,A</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>15</v>
       </c>
@@ -1373,14 +1351,14 @@
         <v>欣[test_capfloor.xlsx]Floor!R10C2IborCoupon,A</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="28"/>
       <c r="B11" s="8" t="str">
         <f>_xll.qlIborCoupon(B6,B7,B4,B6,0,B9)</f>
         <v>欣[test_capfloor.xlsx]Floor!R11C2IborCoupon,A</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="28" t="s">
         <v>37</v>
       </c>
@@ -1388,13 +1366,13 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="28"/>
       <c r="B13" s="8">
         <v>0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>38</v>
       </c>
@@ -1403,7 +1381,7 @@
         <v>欣[test_capfloor.xlsx]Floor!R14C2Floor,A</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>16</v>
       </c>
@@ -1412,7 +1390,7 @@
         <v>欣[test_capfloor.xlsx]Floor!R15C2CashFlow,A</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>18</v>
       </c>
@@ -1421,7 +1399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>19</v>
       </c>
@@ -1430,7 +1408,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>20</v>
       </c>
@@ -1439,7 +1417,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>21</v>
       </c>
@@ -1448,7 +1426,7 @@
         <v>46395</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>22</v>
       </c>
@@ -1457,43 +1435,34 @@
         <v>FLOOR</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Floor!R21C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="8" t="str">
+      <c r="B22" s="8">
         <f>_xll.qlCapFloorAtmRate(B14,B21)</f>
-        <v xml:space="preserve">TypeError: TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\capfloor.py", line 150, in qlCapFloorAtmRate
-    return capfloor.atmRate(discount_curve)
-           ~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 26935, in atmRate
-    return _QuantLib.CapFloor_atmRate(self, discountCurve)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^^^^^^
-TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3.0038607816972797E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B23" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Floor!R23C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>32</v>
       </c>
@@ -1501,7 +1470,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>25</v>
       </c>
@@ -1510,7 +1479,7 @@
         <v>欣[test_capfloor.xlsx]Floor!R25C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>29</v>
       </c>
@@ -1519,16 +1488,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>30</v>
       </c>
       <c r="B27" s="8">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v>4.4068516443390479E-2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlInstrumentNPV(B14,B26)</f>
+        <v>1.8800117125422198</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>17</v>
       </c>
@@ -1537,25 +1506,25 @@
         <v>9.9999999999999995E-8</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B29" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Floor!R29C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>36</v>
       </c>
       <c r="B30" s="8" t="str">
-        <f>_xll.qlConstantOptionletVolatility(B1,"TARGET","Following",0.2,"actual365Fixed")</f>
+        <f>_xll.qlConstantOptionletVolatility(B2,"TARGET","Following",0.2,"actual365Fixed")</f>
         <v>欣[test_capfloor.xlsx]Floor!R30C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>26</v>
       </c>
@@ -1564,7 +1533,7 @@
         <v>欣[test_capfloor.xlsx]Floor!R31C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
         <v>29</v>
       </c>
@@ -1573,25 +1542,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="8">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v>4.4068516443390479E-2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlInstrumentNPV(B14,B32)</f>
+        <v>1.8800117125422198</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B34" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Floor!R34C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>32</v>
       </c>
@@ -1599,7 +1568,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>27</v>
       </c>
@@ -1608,7 +1577,7 @@
         <v>欣[test_capfloor.xlsx]Floor!R36C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
         <v>29</v>
       </c>
@@ -1617,34 +1586,34 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>30</v>
       </c>
       <c r="B38" s="8">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v>4.4068516443390479E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlInstrumentNPV(B14,B37)</f>
+        <v>1.8812663246588561</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B39" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Floor!R39C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B40" s="8" t="str">
-        <f>_xll.qlConstantOptionletVolatility(B1,"TARGET","Following",0.002,"actual365Fixed","normal")</f>
+        <f>_xll.qlConstantOptionletVolatility(B2,"TARGET","Following",0.002,"actual365Fixed","normal")</f>
         <v>欣[test_capfloor.xlsx]Floor!R40C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
         <v>28</v>
       </c>
@@ -1653,7 +1622,7 @@
         <v>欣[test_capfloor.xlsx]Floor!R41C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
         <v>29</v>
       </c>
@@ -1662,13 +1631,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>30</v>
       </c>
       <c r="B43" s="8">
-        <f>_xll.qlInstrumentNPV(B14)</f>
-        <v>4.4068516443390479E-2</v>
+        <f>_xll.qlInstrumentNPV(B14,B42)</f>
+        <v>1.8800117125422198</v>
       </c>
     </row>
   </sheetData>
@@ -1684,15 +1653,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61CB6721-D4A1-4BF9-B717-72F271F45D15}">
   <dimension ref="A1:E45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="57.85546875" customWidth="1"/>
-    <col min="2" max="2" width="82.140625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="36.85546875" style="8" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" style="8"/>
+    <col min="1" max="1" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="82.109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="36.88671875" style="8" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1700,7 +1669,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1709,7 +1678,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>10</v>
       </c>
@@ -1717,7 +1686,7 @@
         <v>46030</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
@@ -1725,7 +1694,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -1734,7 +1703,7 @@
       </c>
       <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
@@ -1742,16 +1711,16 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B8" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Collar!R8C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>34</v>
       </c>
@@ -1760,23 +1729,23 @@
         <v>欣[test_capfloor.xlsx]Collar!R9C2USDLibor,A</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="8" t="str">
-        <f>_xll.qlIborCoupon(B4,B5,B1,B4,0,B9)</f>
+        <f>_xll.qlIborCoupon(B4,B5,B2,B4,0,B9,,,,,,,,B2)</f>
         <v>欣[test_capfloor.xlsx]Collar!R10C2IborCoupon,A</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="28"/>
       <c r="B11" s="8" t="str">
-        <f>_xll.qlIborCoupon(B6,B7,B4,B6,0,B9)</f>
+        <f>_xll.qlIborCoupon(B6,B7,B4,B6,0,B9,,,,,,,,B2)</f>
         <v>欣[test_capfloor.xlsx]Collar!R11C2IborCoupon,A</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="28" t="s">
         <v>35</v>
       </c>
@@ -1784,13 +1753,13 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="13" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="28"/>
       <c r="B13" s="8">
         <v>0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="28" t="s">
         <v>37</v>
       </c>
@@ -1798,13 +1767,13 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="15" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="28"/>
       <c r="B15" s="8">
         <v>0.01</v>
       </c>
     </row>
-    <row r="16" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>39</v>
       </c>
@@ -1813,7 +1782,7 @@
         <v>欣[test_capfloor.xlsx]Collar!R16C2Collar,A</v>
       </c>
     </row>
-    <row r="17" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>16</v>
       </c>
@@ -1822,7 +1791,7 @@
         <v>欣[test_capfloor.xlsx]Collar!R17C2CashFlow,A</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>18</v>
       </c>
@@ -1831,7 +1800,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>19</v>
       </c>
@@ -1840,7 +1809,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="20" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>20</v>
       </c>
@@ -1849,7 +1818,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="21" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>21</v>
       </c>
@@ -1858,7 +1827,7 @@
         <v>46395</v>
       </c>
     </row>
-    <row r="22" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>22</v>
       </c>
@@ -1867,43 +1836,34 @@
         <v>COLLAR</v>
       </c>
     </row>
-    <row r="23" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Collar!R23C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="8" t="str">
+      <c r="B24" s="8">
         <f>_xll.qlCapFloorAtmRate(B16,B23)</f>
-        <v xml:space="preserve">TypeError: TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\capfloor.py", line 150, in qlCapFloorAtmRate
-    return capfloor.atmRate(discount_curve)
-           ~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 26935, in atmRate
-    return _QuantLib.CapFloor_atmRate(self, discountCurve)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^^^^^^
-TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+        <v>3.0038607816972797E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B25" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Collar!R25C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="26" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>32</v>
       </c>
@@ -1911,7 +1871,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="27" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>25</v>
       </c>
@@ -1920,7 +1880,7 @@
         <v>欣[test_capfloor.xlsx]Collar!R27C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="28" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="12" t="s">
         <v>29</v>
       </c>
@@ -1929,61 +1889,43 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="8" t="str">
-        <f>_xll.qlInstrumentNPV(B16)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="8">
+        <f>_xll.qlInstrumentNPV(B16,B28)</f>
+        <v>5.1198820569102951E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="8" t="str">
+      <c r="B30" s="8">
         <f>_xll.qlCapFloorImpliedVolatility(B16,B29,B25,0.2)</f>
-        <v>Error in arg 2 'price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-': Expected float</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B31" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Collar!R31C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="32" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>36</v>
       </c>
       <c r="B32" s="8" t="str">
-        <f>_xll.qlConstantOptionletVolatility(B1,"TARGET","Following",0.2,"actual365Fixed")</f>
+        <f>_xll.qlConstantOptionletVolatility(B2,"TARGET","Following",0.2,"actual365Fixed")</f>
         <v>欣[test_capfloor.xlsx]Collar!R32C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="33" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
         <v>26</v>
       </c>
@@ -1992,7 +1934,7 @@
         <v>欣[test_capfloor.xlsx]Collar!R33C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="34" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
         <v>29</v>
       </c>
@@ -2001,25 +1943,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="8">
-        <f>_xll.qlInstrumentNPV(B16)</f>
-        <v>9.0604094423498536E-5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+        <f>_xll.qlInstrumentNPV(B16,B34)</f>
+        <v>5.1198820569102951E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B36" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Collar!R36C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="37" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>32</v>
       </c>
@@ -2027,7 +1969,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
         <v>27</v>
       </c>
@@ -2036,7 +1978,7 @@
         <v>欣[test_capfloor.xlsx]Collar!R38C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="39" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="12" t="s">
         <v>29</v>
       </c>
@@ -2045,34 +1987,34 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>30</v>
       </c>
       <c r="B40" s="8">
-        <f>_xll.qlInstrumentNPV(B16)</f>
-        <v>9.0604094423498536E-5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+        <f>_xll.qlInstrumentNPV(B16,B39)</f>
+        <v>3.8652710022632174E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B41" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]Collar!R41C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="42" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B42" s="8" t="str">
-        <f>_xll.qlConstantOptionletVolatility(B1,"TARGET","Following",0.002,"actual365Fixed","normal")</f>
+        <f>_xll.qlConstantOptionletVolatility(B2,"TARGET","Following",0.002,"actual365Fixed","normal")</f>
         <v>欣[test_capfloor.xlsx]Collar!R42C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="43" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
         <v>28</v>
       </c>
@@ -2081,7 +2023,7 @@
         <v>欣[test_capfloor.xlsx]Collar!R43C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="44" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="12" t="s">
         <v>29</v>
       </c>
@@ -2090,13 +2032,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>30</v>
       </c>
       <c r="B45" s="8">
-        <f>_xll.qlInstrumentNPV(B16)</f>
-        <v>9.0604094423498536E-5</v>
+        <f>_xll.qlInstrumentNPV(B16,B44)</f>
+        <v>3.8652710022632174E-3</v>
       </c>
     </row>
   </sheetData>
@@ -2113,15 +2055,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A1DD47-423E-4B71-9770-A17F281B15D1}">
   <dimension ref="A1:E51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="57.85546875" customWidth="1"/>
-    <col min="2" max="2" width="55.85546875" style="8" customWidth="1"/>
-    <col min="3" max="3" width="36.85546875" style="8" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" style="8"/>
+    <col min="1" max="1" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="55.88671875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="36.88671875" style="8" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -2129,7 +2071,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2138,7 +2080,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -2146,7 +2088,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>41</v>
       </c>
@@ -2154,16 +2096,16 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B6" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R6C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
         <v>42</v>
       </c>
@@ -2172,7 +2114,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R7C2USDLibor,A</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -2180,7 +2122,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>44</v>
       </c>
@@ -2188,7 +2130,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -2196,13 +2138,13 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B11" s="7"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -2210,7 +2152,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -2218,7 +2160,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -2226,7 +2168,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>50</v>
       </c>
@@ -2234,7 +2176,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -2242,19 +2184,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>52</v>
       </c>
       <c r="B17" s="7"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>53</v>
       </c>
       <c r="B18" s="7"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -2262,7 +2204,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>55</v>
       </c>
@@ -2270,21 +2212,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>61</v>
       </c>
       <c r="B22" s="8" t="str">
-        <f>_xll.qlMakeCapFloor(B4,B5,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16,B17,B18,B19,B20)</f>
+        <f>_xll.qlMakeCapFloor(B4,B5,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16,B17,B18,B19,B20,,B2)</f>
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R22C2CapFloor,A</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
         <v>16</v>
       </c>
@@ -2293,7 +2235,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R23C2CashFlow,A</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>18</v>
       </c>
@@ -2302,7 +2244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>19</v>
       </c>
@@ -2311,7 +2253,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>20</v>
       </c>
@@ -2320,7 +2262,7 @@
         <v>45670</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>21</v>
       </c>
@@ -2329,7 +2271,7 @@
         <v>46035</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>22</v>
       </c>
@@ -2338,43 +2280,34 @@
         <v>FLOOR</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>24</v>
       </c>
       <c r="B29" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R29C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="8" t="str">
+      <c r="B30" s="8">
         <f>_xll.qlCapFloorAtmRate(B22,B29)</f>
-        <v xml:space="preserve">TypeError: TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\capfloor.py", line 150, in qlCapFloorAtmRate
-    return capfloor.atmRate(discount_curve)
-           ~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 26935, in atmRate
-    return _QuantLib.CapFloor_atmRate(self, discountCurve)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^^^^^^^^^
-TypeError: in method 'CapFloor_atmRate', argument 2 of type 'YieldTermStructure const &amp;'
-</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+        <v>2.9700276978901811E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B31" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R31C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>32</v>
       </c>
@@ -2382,7 +2315,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
         <v>25</v>
       </c>
@@ -2391,7 +2324,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R33C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
         <v>29</v>
       </c>
@@ -2400,52 +2333,34 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="8" t="str">
-        <f>_xll.qlInstrumentNPV(B22)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="8">
+        <f>_xll.qlInstrumentNPV(B22,B34)</f>
+        <v>4.633076994730075E-4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="8" t="str">
+      <c r="B36" s="8">
         <f>_xll.qlCapFloorImpliedVolatility(B22,B35,B31,0.2)</f>
-        <v>Error in arg 2 'price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-': Expected float</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B37" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R37C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
         <v>36</v>
       </c>
@@ -2454,7 +2369,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R38C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
         <v>26</v>
       </c>
@@ -2463,7 +2378,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R39C2BlackCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="12" t="s">
         <v>29</v>
       </c>
@@ -2472,34 +2387,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="8" t="str">
-        <f>_xll.qlInstrumentNPV(B22)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B41" s="8">
+        <f>_xll.qlInstrumentNPV(B22,B40)</f>
+        <v>1.339625003165777</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B42" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R42C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
         <v>32</v>
       </c>
@@ -2507,7 +2413,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
         <v>27</v>
       </c>
@@ -2516,7 +2422,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R44C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="12" t="s">
         <v>29</v>
       </c>
@@ -2525,25 +2431,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>30</v>
       </c>
       <c r="B46" s="8">
-        <f>_xll.qlInstrumentNPV(B22)</f>
-        <v>1.0860189240505816E-5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlInstrumentNPV(B22,B45)</f>
+        <v>0.48196197214187886</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B47" s="8" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Act/365")</f>
+        <f>_xll.qlFlatForward(B2,0.03,"Act/365")</f>
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R47C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" s="9" t="s">
         <v>36</v>
       </c>
@@ -2552,7 +2458,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R48C2OptionletVolatilityStructureHandle,A</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="14" t="s">
         <v>28</v>
       </c>
@@ -2561,7 +2467,7 @@
         <v>欣[test_capfloor.xlsx]MakeCapFloor!R49C2BachelierCapFloorEngine,A</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
         <v>29</v>
       </c>
@@ -2570,22 +2476,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>30</v>
       </c>
-      <c r="B51" s="8" t="str">
-        <f>_xll.qlInstrumentNPV(B22)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\instruments.py", line 18, in qlInstrumentNPV
-    return instrument.NPV()
-           ~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 16448, in NPV
-    return _QuantLib.Instrument_NPV(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: null pricing engine
-</v>
+      <c r="B51" s="8">
+        <f>_xll.qlInstrumentNPV(B22,B50)</f>
+        <v>1.339625003165777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>